<commit_message>
feat: Agent 6.9 작업 브랜치 반영
</commit_message>
<xml_diff>
--- a/data/market_excel/market_final_DB하이텍.xlsx
+++ b/data/market_excel/market_final_DB하이텍.xlsx
@@ -510,47 +510,33 @@
           <t>보유</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v>35</v>
+      </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>DB하이텍 분석 중 LLM 호출 오류가 발생해 fallback 결과를 반환합니다.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>IDM/제조/메모리</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
+          <t>DB하이텍은 강한 주가 상승 모멘텀을 보이고 있으나, 거시 경제 불확실성과 경쟁 구도 불명확성으로 인해 '보유' 의견을 제시합니다. 아날로그 반도체 전문 파운드리 시장에서의 경쟁력은 긍정적입니다.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -624,25 +610,27 @@
           <t>보유</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v>35</v>
+      </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>DB하이텍 분석 중 LLM 호출 오류가 발생해 fallback 결과를 반환합니다.</t>
+          <t>DB하이텍은 강한 주가 상승 모멘텀을 보이고 있으나, 거시 경제 불확실성과 경쟁 구도 불명확성으로 인해 '보유' 의견을 제시합니다. 아날로그 반도체 전문 파운드리 시장에서의 경쟁력은 긍정적입니다.</t>
         </is>
       </c>
     </row>
@@ -725,7 +713,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IDM/제조/메모리</t>
+          <t>후공정/패키징/테스트</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -742,12 +730,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>높음</t>
+          <t>중간</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DB하이텍은 8인치 순수 파운드리 기업으로 다품종 소량 생산이 가능하며, 특히 Analog 반도체 전문성을 바탕으로 고객 맞춤형 공정 기술을 제공하고 있다.</t>
+          <t>세계 유수의 반도체 업체들에게 최첨단 반도체 패키징 솔루션을 제공하여 업계에서 신뢰받는 기업으로 자리 잡고 있습니다.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -757,22 +745,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>사업보고서에서 DB하이텍이 비메모리 반도체의 파운드리 사업을 주요 사업으로 영위한다고 명시되어 있다.</t>
+          <t>사업 개요에서 반도체 조립 및 테스트 제품을 주력으로 생산하고 있다고 명시되어 있습니다.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>20241114001868</t>
+          <t>20241113000459</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-05-20T11:14:53.681949</t>
+          <t>2026-05-25T11:09:12.756789</t>
         </is>
       </c>
     </row>
@@ -931,7 +919,7 @@
         <v>180.5</v>
       </c>
       <c r="G2" t="n">
-        <v>134.8</v>
+        <v>143.9</v>
       </c>
     </row>
     <row r="3">
@@ -946,19 +934,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>533.7</v>
+        <v>528.8</v>
       </c>
       <c r="D3" t="n">
-        <v>619.5</v>
+        <v>680.1</v>
       </c>
       <c r="E3" t="n">
-        <v>548.6</v>
+        <v>556.6</v>
       </c>
       <c r="F3" t="n">
-        <v>795.3</v>
+        <v>683.7</v>
       </c>
       <c r="G3" t="n">
-        <v>1896.6</v>
+        <v>1913.6</v>
       </c>
     </row>
     <row r="4">
@@ -979,13 +967,13 @@
         <v>293.4</v>
       </c>
       <c r="E4" t="n">
-        <v>224.9</v>
+        <v>224.8</v>
       </c>
       <c r="F4" t="n">
-        <v>495.2</v>
+        <v>455.2</v>
       </c>
       <c r="G4" t="n">
-        <v>1885.4</v>
+        <v>1527.9</v>
       </c>
     </row>
     <row r="5">
@@ -1012,7 +1000,7 @@
         <v>102.3</v>
       </c>
       <c r="G5" t="n">
-        <v>115.6</v>
+        <v>123.3</v>
       </c>
     </row>
     <row r="6">
@@ -1033,13 +1021,13 @@
         <v>406</v>
       </c>
       <c r="E6" t="n">
-        <v>500.7</v>
+        <v>481</v>
       </c>
       <c r="F6" t="n">
-        <v>429.9</v>
+        <v>464.2</v>
       </c>
       <c r="G6" t="n">
-        <v>551.3</v>
+        <v>469.4</v>
       </c>
     </row>
     <row r="7">
@@ -1084,16 +1072,16 @@
         <v>665</v>
       </c>
       <c r="D8" t="n">
-        <v>570</v>
+        <v>578.8</v>
       </c>
       <c r="E8" t="n">
-        <v>548.6</v>
+        <v>533.8</v>
       </c>
       <c r="F8" t="n">
         <v>605.9</v>
       </c>
       <c r="G8" t="n">
-        <v>851.1</v>
+        <v>750.7</v>
       </c>
     </row>
     <row r="9">
@@ -1111,16 +1099,16 @@
         <v>520</v>
       </c>
       <c r="D9" t="n">
-        <v>577.1</v>
+        <v>602.6</v>
       </c>
       <c r="E9" t="n">
-        <v>602.9</v>
+        <v>631</v>
       </c>
       <c r="F9" t="n">
-        <v>722.9</v>
+        <v>727.8</v>
       </c>
       <c r="G9" t="n">
-        <v>832</v>
+        <v>822.4</v>
       </c>
     </row>
     <row r="10">
@@ -1147,7 +1135,7 @@
         <v>61.5</v>
       </c>
       <c r="G10" t="n">
-        <v>70.3</v>
+        <v>71.3</v>
       </c>
     </row>
     <row r="11">
@@ -1165,16 +1153,16 @@
         <v>566.1</v>
       </c>
       <c r="D11" t="n">
-        <v>551.6</v>
+        <v>558.4</v>
       </c>
       <c r="E11" t="n">
-        <v>473.6</v>
+        <v>507.1</v>
       </c>
       <c r="F11" t="n">
-        <v>676.1</v>
+        <v>675</v>
       </c>
       <c r="G11" t="n">
-        <v>803.6</v>
+        <v>807.1</v>
       </c>
     </row>
     <row r="12">
@@ -1219,16 +1207,16 @@
         <v>481.6</v>
       </c>
       <c r="D13" t="n">
-        <v>483.4</v>
+        <v>490.2</v>
       </c>
       <c r="E13" t="n">
-        <v>535.7</v>
+        <v>533.5</v>
       </c>
       <c r="F13" t="n">
-        <v>681.1</v>
+        <v>650.8</v>
       </c>
       <c r="G13" t="n">
-        <v>796.7</v>
+        <v>796.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>